<commit_message>
Prevent silent loading failures when Tradebook Template is locked or open in Excel
</commit_message>
<xml_diff>
--- a/Tradebook Template.xlsx
+++ b/Tradebook Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="58" documentId="11_B8E6E54BA230E35AD1C0AFADF073B256A24125FE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46D75A32-2695-4048-88FC-00D86510DD5B}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="11_B8E6E54BA230E35AD1C0AFADF073B256A24125FE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6348F31-F2B5-4DB8-9065-716907BEEF85}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="76">
   <si>
     <t>Symbol</t>
   </si>
@@ -81,70 +81,184 @@
     <t>buy</t>
   </si>
   <si>
-    <t>SOLARINDS</t>
-  </si>
-  <si>
-    <t>INE343H01029</t>
-  </si>
-  <si>
-    <t>TDPOWERSYS</t>
-  </si>
-  <si>
-    <t>INE419M01027</t>
-  </si>
-  <si>
-    <t>GVT&amp;D</t>
-  </si>
-  <si>
-    <t>INE200A01026</t>
-  </si>
-  <si>
-    <t>2026-06-04T11:45:35</t>
-  </si>
-  <si>
     <t>BSE</t>
   </si>
   <si>
     <t>A</t>
   </si>
   <si>
-    <t>2026-06-04T11:48:33</t>
-  </si>
-  <si>
-    <t>2026-06-04T11:55:25</t>
-  </si>
-  <si>
-    <t>2026-06-04</t>
-  </si>
-  <si>
-    <t>205454282</t>
-  </si>
-  <si>
-    <t>1100000050186797</t>
-  </si>
-  <si>
-    <t>5961700</t>
-  </si>
-  <si>
-    <t>1780550482158604643</t>
-  </si>
-  <si>
-    <t>5962300</t>
-  </si>
-  <si>
-    <t>5962100</t>
-  </si>
-  <si>
-    <t>5961900</t>
-  </si>
-  <si>
-    <t>5962500</t>
-  </si>
-  <si>
-    <t>604868027</t>
-  </si>
-  <si>
-    <t>1300000047270644</t>
+    <t>SUNPHARMA</t>
+  </si>
+  <si>
+    <t>INE044A01036</t>
+  </si>
+  <si>
+    <t>2026-06-05</t>
+  </si>
+  <si>
+    <t>sell</t>
+  </si>
+  <si>
+    <t>607608623</t>
+  </si>
+  <si>
+    <t>1300000080435508</t>
+  </si>
+  <si>
+    <t>2026-06-05T14:11:19</t>
+  </si>
+  <si>
+    <t>607608625</t>
+  </si>
+  <si>
+    <t>607608624</t>
+  </si>
+  <si>
+    <t>GPIL</t>
+  </si>
+  <si>
+    <t>INE177H01039</t>
+  </si>
+  <si>
+    <t>207863043</t>
+  </si>
+  <si>
+    <t>1100000081623474</t>
+  </si>
+  <si>
+    <t>2026-06-05T14:11:52</t>
+  </si>
+  <si>
+    <t>207863041</t>
+  </si>
+  <si>
+    <t>207863052</t>
+  </si>
+  <si>
+    <t>207863050</t>
+  </si>
+  <si>
+    <t>207863046</t>
+  </si>
+  <si>
+    <t>207863042</t>
+  </si>
+  <si>
+    <t>207863051</t>
+  </si>
+  <si>
+    <t>207863049</t>
+  </si>
+  <si>
+    <t>207863047</t>
+  </si>
+  <si>
+    <t>207863048</t>
+  </si>
+  <si>
+    <t>207863045</t>
+  </si>
+  <si>
+    <t>207863044</t>
+  </si>
+  <si>
+    <t>TATATECH</t>
+  </si>
+  <si>
+    <t>INE142M01025</t>
+  </si>
+  <si>
+    <t>8566100</t>
+  </si>
+  <si>
+    <t>1780650791219152130</t>
+  </si>
+  <si>
+    <t>2026-06-05T14:54:16</t>
+  </si>
+  <si>
+    <t>LAURUSLABS</t>
+  </si>
+  <si>
+    <t>INE947Q01028</t>
+  </si>
+  <si>
+    <t>6439100</t>
+  </si>
+  <si>
+    <t>1780646107540983562</t>
+  </si>
+  <si>
+    <t>2026-06-05T14:55:18</t>
+  </si>
+  <si>
+    <t>BALAMINES</t>
+  </si>
+  <si>
+    <t>INE050E01027</t>
+  </si>
+  <si>
+    <t>6653160</t>
+  </si>
+  <si>
+    <t>1000000077505165</t>
+  </si>
+  <si>
+    <t>2026-06-05T14:58:19</t>
+  </si>
+  <si>
+    <t>6653157</t>
+  </si>
+  <si>
+    <t>6653161</t>
+  </si>
+  <si>
+    <t>6653158</t>
+  </si>
+  <si>
+    <t>6653159</t>
+  </si>
+  <si>
+    <t>7090800</t>
+  </si>
+  <si>
+    <t>1780651635390503732</t>
+  </si>
+  <si>
+    <t>2026-06-05T15:21:19</t>
+  </si>
+  <si>
+    <t>ZENTEC</t>
+  </si>
+  <si>
+    <t>INE251B01027</t>
+  </si>
+  <si>
+    <t>609856815</t>
+  </si>
+  <si>
+    <t>1300000099844907</t>
+  </si>
+  <si>
+    <t>2026-06-05T15:24:23</t>
+  </si>
+  <si>
+    <t>609856816</t>
+  </si>
+  <si>
+    <t>EXIDEIND</t>
+  </si>
+  <si>
+    <t>INE302A01020</t>
+  </si>
+  <si>
+    <t>210316684</t>
+  </si>
+  <si>
+    <t>1100000100822022</t>
+  </si>
+  <si>
+    <t>2026-06-05T15:27:06</t>
   </si>
 </sst>
 </file>
@@ -531,43 +645,43 @@
     </row>
     <row r="2" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="I2" s="3" t="b">
         <v>0</v>
       </c>
       <c r="J2" s="4">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K2" s="4">
-        <v>5100</v>
+        <v>1790.5</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.25">
@@ -578,37 +692,37 @@
         <v>19</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>1</v>
+      </c>
+      <c r="K3" s="4">
+        <v>1790.3</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="M3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J3" s="4">
-        <v>18</v>
-      </c>
-      <c r="K3" s="4">
-        <v>1350.75</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
@@ -619,296 +733,999 @@
         <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4">
+        <v>15</v>
+      </c>
+      <c r="K4" s="4">
+        <v>1790.3</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="3" t="s">
+      <c r="N4" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J4" s="4">
-        <v>3</v>
-      </c>
-      <c r="K4" s="4">
-        <v>1351</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I5" s="3" t="b">
         <v>0</v>
       </c>
       <c r="J5" s="4">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="K5" s="4">
-        <v>1350.85</v>
+        <v>280.75</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="M5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N5" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I6" s="3" t="b">
         <v>0</v>
       </c>
       <c r="J6" s="4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K6" s="4">
-        <v>1350.8</v>
+        <v>280.75</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="M6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N6" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="N6" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4">
         <v>19</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J7" s="4">
-        <v>5</v>
-      </c>
       <c r="K7" s="4">
-        <v>1351.1</v>
+        <v>280.64999999999998</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N7" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" s="4">
+        <v>30</v>
+      </c>
+      <c r="K8" s="4">
+        <v>280.64999999999998</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4">
+        <v>30</v>
+      </c>
+      <c r="K9" s="4">
+        <v>280.7</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4">
+        <v>30</v>
+      </c>
+      <c r="K10" s="4">
+        <v>280.75</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N10" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4">
+        <v>32</v>
+      </c>
+      <c r="K11" s="4">
+        <v>280.64999999999998</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4">
+        <v>88</v>
+      </c>
+      <c r="K12" s="4">
+        <v>280.7</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I13" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J13" s="4">
+        <v>9</v>
+      </c>
+      <c r="K13" s="4">
+        <v>280.7</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N13" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I14" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14" s="4">
+        <v>9</v>
+      </c>
+      <c r="K14" s="4">
+        <v>280.7</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I15" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4">
+        <v>10</v>
+      </c>
+      <c r="K15" s="4">
+        <v>280.75</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I16" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J16" s="4">
+        <v>9</v>
+      </c>
+      <c r="K16" s="4">
+        <v>280.75</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="F17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="3" t="s">
+      <c r="H17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J8" s="4">
-        <v>2</v>
-      </c>
-      <c r="K8" s="4">
-        <v>18502</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="N8" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-    </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-    </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-    </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-    </row>
-    <row r="17" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-    </row>
-    <row r="18" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-    </row>
-    <row r="19" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-    </row>
-    <row r="20" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-    </row>
-    <row r="21" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-    </row>
-    <row r="22" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-    </row>
-    <row r="23" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-    </row>
-    <row r="24" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-    </row>
-    <row r="25" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-    </row>
-    <row r="26" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-    </row>
-    <row r="27" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-    </row>
-    <row r="28" spans="10:11" x14ac:dyDescent="0.25">
+      <c r="I17" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J17" s="4">
+        <v>65</v>
+      </c>
+      <c r="K17" s="4">
+        <v>767.25</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="N17" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I18" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J18" s="4">
+        <v>34</v>
+      </c>
+      <c r="K18" s="4">
+        <v>1449.5</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="N18" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J19" s="4">
+        <v>11</v>
+      </c>
+      <c r="K19" s="4">
+        <v>2027.9</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="M19" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="N19" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I20" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J20" s="4">
+        <v>1</v>
+      </c>
+      <c r="K20" s="4">
+        <v>2027.6</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="N20" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J21" s="4">
+        <v>29</v>
+      </c>
+      <c r="K21" s="4">
+        <v>2028</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="N21" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J22" s="4">
+        <v>4</v>
+      </c>
+      <c r="K22" s="4">
+        <v>2027.6</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="M22" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="N22" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J23" s="4">
+        <v>4</v>
+      </c>
+      <c r="K23" s="4">
+        <v>2027.8</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="M23" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="N23" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B24" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I24" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J24" s="4">
+        <v>34</v>
+      </c>
+      <c r="K24" s="4">
+        <v>1446.35</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="N24" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B25" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I25" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J25" s="4">
+        <v>5</v>
+      </c>
+      <c r="K25" s="4">
+        <v>1817.3</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="N25" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B26" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I26" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J26" s="4">
+        <v>9</v>
+      </c>
+      <c r="K26" s="4">
+        <v>1817.8</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="N26" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B27" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I27" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J27" s="4">
+        <v>125</v>
+      </c>
+      <c r="K27" s="4">
+        <v>399.6</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="M27" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="N27" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="10:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:14" x14ac:dyDescent="0.25">
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
     </row>
-    <row r="30" spans="10:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
     </row>
-    <row r="31" spans="10:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
     </row>
-    <row r="32" spans="10:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:14" x14ac:dyDescent="0.25">
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
     </row>

</xml_diff>